<commit_message>
Final commit for the project, removed unnecesarry files, and fixed 2 hour slot scheduling
</commit_message>
<xml_diff>
--- a/output/unscheduled_courses.xlsx
+++ b/output/unscheduled_courses.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -474,50 +474,75 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B1-CS366</t>
+          <t>CS307</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>CSE</t>
+          <t>DSAI</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>LEC</t>
+          <t>LAB</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>No suitable room found (Needs 200 capacity)</t>
+          <t>No computer lab available (Needs 80 capacity)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>EC161</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DSAI</t>
+          <t>Common_7th</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>LAB</t>
+          <t>LEC</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No computer lab available (Needs 110 capacity)</t>
+          <t>Could not schedule basket B2 (Needs 200 capacity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Common_7th</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>LEC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Could not schedule basket B4 (Needs 200 capacity)</t>
         </is>
       </c>
     </row>

</xml_diff>